<commit_message>
All changes done after meeting except Multiple SSC selection on NOS add
</commit_message>
<xml_diff>
--- a/public/uploads/sample/bulk_nos_pc_sample_file.xlsx
+++ b/public/uploads/sample/bulk_nos_pc_sample_file.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\projects\uatassmt\public\uploads\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9533032D-D38A-4769-BF5A-26D1DD82B3E5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0734D2B-2889-4B9F-9FD1-7DE013F633A5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32760" yWindow="32760" windowWidth="20385" windowHeight="7950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
   <si>
     <t>PC_ID</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>15</t>
+  </si>
+  <si>
+    <t>Project_Marks</t>
   </si>
 </sst>
 </file>
@@ -452,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultColWidth="12.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" style="1" customWidth="1"/>
@@ -469,7 +472,7 @@
     <col min="12" max="16384" width="12.28515625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -494,8 +497,11 @@
       <c r="H1" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="I1" s="2" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
@@ -520,8 +526,11 @@
       <c r="H2" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="I2" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -546,8 +555,11 @@
       <c r="H3" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="I3" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
@@ -572,8 +584,11 @@
       <c r="H4" s="1" t="s">
         <v>23</v>
       </c>
+      <c r="I4" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
@@ -596,6 +611,9 @@
         <v>21</v>
       </c>
       <c r="H5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>